<commit_message>
Remove duplicate Tailwind directives in index.css
</commit_message>
<xml_diff>
--- a/backend/uploads/individuales/EMERGENCIA/1/Planilla_1_EMERGENCIA.xlsx
+++ b/backend/uploads/individuales/EMERGENCIA/1/Planilla_1_EMERGENCIA.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="44">
   <si>
     <t>CENTRO CLINICO QUIRÚRGICO AMBULATORIO HOSPITAL DEL DÍA CHIMBACALLE</t>
   </si>
@@ -116,9 +116,6 @@
     <t>3432620068050</t>
   </si>
   <si>
-    <t>GUANTES DE LATEX, TALLA PEQUEÑO</t>
-  </si>
-  <si>
     <t>EM09-38</t>
   </si>
   <si>
@@ -152,19 +149,13 @@
     <t>DOCUMENTO DE IDENTIDAD:</t>
   </si>
   <si>
-    <t>1234567890</t>
-  </si>
-  <si>
     <t xml:space="preserve">CARGO: </t>
   </si>
   <si>
-    <t>ANALISTA - FACTURACIÓN</t>
+    <t>RESPONSABLE DE FACTURACION</t>
   </si>
   <si>
     <t>Econ. Ximena Cobos</t>
-  </si>
-  <si>
-    <t>1324567890</t>
   </si>
   <si>
     <t>DIRECTOR ADMINISTRATIVO</t>
@@ -1192,7 +1183,7 @@
       <c r="E6" s="19"/>
       <c r="F6" s="19"/>
       <c r="G6" s="20">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="H6" s="21"/>
       <c r="I6" s="22"/>
@@ -1269,13 +1260,13 @@
         <v>17</v>
       </c>
       <c r="C11" s="31">
-        <v>45884</v>
+        <v>46006</v>
       </c>
       <c r="D11" s="30" t="s">
         <v>18</v>
       </c>
       <c r="E11" s="31">
-        <v>45884</v>
+        <v>46006</v>
       </c>
       <c r="F11" s="30"/>
       <c r="G11" s="30"/>
@@ -1313,13 +1304,13 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="36">
-        <v>45884</v>
+        <v>46006</v>
       </c>
       <c r="B13" s="36" t="s">
         <v>28</v>
       </c>
       <c r="C13" s="36" t="s">
-        <v>29</v>
+        <v>11</v>
       </c>
       <c r="D13" s="36">
         <v>4</v>
@@ -1331,7 +1322,7 @@
         <v>0.28</v>
       </c>
       <c r="G13" s="36" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H13" s="36">
         <v>100</v>
@@ -1342,13 +1333,13 @@
     </row>
     <row r="14" ht="37.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="36">
-        <v>45884</v>
+        <v>46006</v>
       </c>
       <c r="B14" s="36" t="s">
+        <v>30</v>
+      </c>
+      <c r="C14" s="36" t="s">
         <v>31</v>
-      </c>
-      <c r="C14" s="36" t="s">
-        <v>32</v>
       </c>
       <c r="D14" s="36">
         <v>3</v>
@@ -1360,7 +1351,7 @@
         <v>4.02</v>
       </c>
       <c r="G14" s="36" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H14" s="36">
         <v>100</v>
@@ -1371,13 +1362,13 @@
     </row>
     <row r="15" ht="39" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="36">
-        <v>45884</v>
+        <v>46006</v>
       </c>
       <c r="B15" s="36" t="s">
+        <v>33</v>
+      </c>
+      <c r="C15" s="36" t="s">
         <v>34</v>
-      </c>
-      <c r="C15" s="36" t="s">
-        <v>35</v>
       </c>
       <c r="D15" s="36">
         <v>1</v>
@@ -1389,7 +1380,7 @@
         <v>20.57</v>
       </c>
       <c r="G15" s="36" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H15" s="36">
         <v>100</v>
@@ -1818,11 +1809,11 @@
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" s="39" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B54" s="39"/>
       <c r="C54" s="40" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D54" s="41"/>
       <c r="E54" s="41"/>
@@ -1891,10 +1882,10 @@
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" s="47"/>
       <c r="B60" s="50" t="s">
+        <v>37</v>
+      </c>
+      <c r="C60" s="51" t="s">
         <v>38</v>
-      </c>
-      <c r="C60" s="51" t="s">
-        <v>39</v>
       </c>
       <c r="D60" s="52"/>
       <c r="E60" s="53"/>
@@ -1906,10 +1897,10 @@
     <row r="61" ht="25.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" s="47"/>
       <c r="B61" s="55" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C61" s="56" t="s">
-        <v>41</v>
+        <v>11</v>
       </c>
       <c r="D61" s="53"/>
       <c r="E61" s="53"/>
@@ -1921,10 +1912,10 @@
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" s="47"/>
       <c r="B62" s="57" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C62" s="58" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D62" s="53"/>
       <c r="E62" s="53"/>
@@ -1958,10 +1949,10 @@
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65" s="47"/>
       <c r="B65" s="50" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C65" s="51" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D65" s="53"/>
       <c r="E65" s="53"/>
@@ -1973,10 +1964,10 @@
     <row r="66" ht="25.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A66" s="47"/>
       <c r="B66" s="55" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C66" s="56" t="s">
-        <v>45</v>
+        <v>11</v>
       </c>
       <c r="D66" s="53"/>
       <c r="E66" s="53"/>
@@ -1988,10 +1979,10 @@
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A67" s="47"/>
       <c r="B67" s="57" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C67" s="58" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D67" s="53"/>
       <c r="E67" s="53"/>

</xml_diff>